<commit_message>
Added Faker API to implement Data Driven Testing using Faker Library. And also added Date and Time Util.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/PhoenixTestData.xlsx
+++ b/src/test/resources/testdata/PhoenixTestData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="4">
   <si>
     <t>username</t>
   </si>
@@ -35,13 +35,10 @@
     <t>password</t>
   </si>
   <si>
-    <t>iamuser1</t>
+    <t>admin</t>
   </si>
   <si>
-    <t>iamuser2</t>
-  </si>
-  <si>
-    <t>iamuser3</t>
+    <t>password123</t>
   </si>
 </sst>
 </file>
@@ -1005,23 +1002,23 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" ht="18" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" ht="18" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>